<commit_message>
Update: Threat Alert Report - 2026-05-21 01:38
</commit_message>
<xml_diff>
--- a/excel_routes/route_CAI_YNB_threats.xlsx
+++ b/excel_routes/route_CAI_YNB_threats.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -459,7 +459,7 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -537,13 +537,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>4783</v>
+        <v>4855</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4936</v>
+        <v>5011</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-153</v>
+        <v>-156</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -556,7 +556,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -568,7 +568,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>20-JUN-26</t>
+          <t>06-JUN-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -582,13 +582,13 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>7837</v>
+        <v>8748</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9050</v>
+        <v>9187</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-1213</v>
+        <v>-439</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>30</v>
@@ -601,415 +601,10 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>EGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>27-JUN-26</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>SM-447</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-103</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>7837</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>9050</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>-1213</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>EGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>01-AUG-26</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>SM-447</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-103</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>9970</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>11128</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>-1158</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>EGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>04-AUG-26</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>SM-441</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-103</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>9970</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>11128</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>-1158</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>EGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>08-AUG-26</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>SM-447</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-103</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>10668</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>11128</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>-460</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>EGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>15-AUG-26</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>SM-447</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-103</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>10668</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>12299</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>-1631</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>EGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>25-AUG-26</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>SM-441</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-103</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>10668</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>11128</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>-460</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>EGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>01-SEP-26</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>SM-441</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-103</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>9970</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>11128</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>-1158</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>EGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>05-SEP-26</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>SM-447</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-103</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>9970</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>11128</v>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>-1158</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>EGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>08-SEP-26</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>SM-441</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-103</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>9970</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>11128</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>-1158</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>EGP</t>
         </is>

</xml_diff>